<commit_message>
feat(FRUKI): adiciona aba V&V — cenários de teste e evidências
Nova aba na planilha de gestão com 15 cenários Gherkin (6 Pacote 1 +
9 PF24), 11 ciclos de execução com defeitos e resoluções, e resumo
de cobertura (100% aprovação em ambos os pacotes), extraídos de
VV-FRUKI01-001 e VV-FRUKI01-002.

https://claude.ai/code/session_011KXfcc9u9SbkrrmomU4zNq
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/RAC-FRUKI01-002_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/RAC-FRUKI01-002_Planilha-de-Gestao-do-Projeto.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Riscos" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Medição" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="GQA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="V&amp;V — Testes" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,8 +68,47 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B7A1B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00856404"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -120,8 +160,38 @@
         <fgColor rgb="00D6EDDF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A5276"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -143,11 +213,25 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -187,6 +271,51 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5666,8 +5795,1398 @@
   <mergeCells count="5">
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A37:E37"/>
     <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A37:E37"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>V&amp;V — Cenários de Teste e Evidências · SuperApp Fruki</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Referências: VV-FRUKI01-001 (Pacote 1) | VV-FRUKI01-002 (Pacote Final 24) | Processo: PRO-VV-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>1. CICLOS DE EXECUÇÃO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Pacote</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Ciclo</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Módulo / Escopo</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>Itens Verificados</t>
+        </is>
+      </c>
+      <c r="E5" s="16" t="inlineStr">
+        <is>
+          <t>Defeitos</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>Resolução</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Situação</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Sprint 1 — Desenvolvimento</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Módulo Metas/RV — telas e APIs</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>RF-01 a RF-04, RNF-01 a RNF-04</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>2 (duplicação famílias API; latência ~3,10 s)</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Tratados no front-end antes do piloto</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Jul/2025</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>Piloto (vendedores reais)</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>Fluxo completo — Metas, Indicadores, RV</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="inlineStr">
+        <is>
+          <t>Todos os RFs — cenários reais</t>
+        </is>
+      </c>
+      <c r="E7" s="21" t="inlineStr">
+        <is>
+          <t>2 (duplicação residual; positivação inconsistente)</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>Corrigidos antes do aceite (Ago/2025)</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
+        <is>
+          <t>05/08/2025</t>
+        </is>
+      </c>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Revisão de PR — Jardel</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>Código-fonte completo</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Todos os RFs + código</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Ago/2025</t>
+        </is>
+      </c>
+      <c r="H8" s="18" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Aceite final</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>Todos os módulos do Pacote 1</t>
+        </is>
+      </c>
+      <c r="D9" s="21" t="inlineStr">
+        <is>
+          <t>Todos os RFs</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F9" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>Set/2025</t>
+        </is>
+      </c>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Sprint 1</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>Pedidos Não Alocados</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="inlineStr">
+        <is>
+          <t>RF-05 a RF-08</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>1 (formato não padronizado da API de pedidos)</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Normalização em pedidosNaoAlocadosService.ts</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>Out/2025</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>Revisão PR #57</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>Módulo Pedidos Não Alocados — código</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
+        <is>
+          <t>Padrões, performance, autenticação</t>
+        </is>
+      </c>
+      <c r="E11" s="21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>25/10/2025</t>
+        </is>
+      </c>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="inlineStr">
+        <is>
+          <t>Sprint 2</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>RF-09 a RF-11</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Módulo entregue conforme protótipo</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>Nov/2025</t>
+        </is>
+      </c>
+      <c r="H12" s="18" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>Revisão PR — Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>Código do módulo Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="D13" s="21" t="inlineStr">
+        <is>
+          <t>Padrões, performance, integração</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>Nov/2025</t>
+        </is>
+      </c>
+      <c r="H13" s="20" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>PDV / Rota PDV</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>RF-12 a RF-14</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>1 (API Rota PDV recebida só em 08/01/2026)</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>Desenvolvimento paralelo da UI; integração Jan/2026</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>Dez/2025–Jan/2026</t>
+        </is>
+      </c>
+      <c r="H14" s="18" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>Build AAB v2.0</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>Todos os módulos — build de produção</t>
+        </is>
+      </c>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>RNF-01, RNF-03</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>AAB gerado e entregue para publicação</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>Jan/2026</t>
+        </is>
+      </c>
+      <c r="H15" s="20" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>Aceite final</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>Todos os módulos do PF24</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>RF-05 a RF-14</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Aceite formal via Microsoft Teams</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>15/01/2026</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>✅ Concluído</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>2. CENÁRIOS DE TESTE — RESULTADOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>Pacote</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Módulo</t>
+        </is>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Cenário</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>Pré-condição / Ação</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="G20" s="16" t="inlineStr">
+        <is>
+          <t>Evidência</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>Situação</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="35" customHeight="1">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>Metas por Família</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="inlineStr">
+        <is>
+          <t>Visualizar metas de volume por família</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E21" s="21" t="inlineStr">
+        <is>
+          <t>Vendedor autenticado acessa tela de Metas</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr">
+        <is>
+          <t>Lista de famílias c/ volume real, meta e % atingimento</t>
+        </is>
+      </c>
+      <c r="G21" s="21" t="inlineStr">
+        <is>
+          <t>APK piloto 05/08/2025 — validado por Cecília</t>
+        </is>
+      </c>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="35" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Metas por Família</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>API retorna famílias duplicadas</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="inlineStr">
+        <is>
+          <t>API retorna registros duplicados para mesma família</t>
+        </is>
+      </c>
+      <c r="F22" s="19" t="inlineStr">
+        <is>
+          <t>Apenas um registro por família exibido; ordenação mantida</t>
+        </is>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>Identificado no piloto; corrigido e revalidado Ago/2025</t>
+        </is>
+      </c>
+      <c r="H22" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="35" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>Metas por Família</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>API demora mais de 3 segundos</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="E23" s="21" t="inlineStr">
+        <is>
+          <t>Resposta da API leva mais de 1 segundo</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr">
+        <is>
+          <t>Skeleton screen exibido; dados aparecem após carregamento</t>
+        </is>
+      </c>
+      <c r="G23" s="21" t="inlineStr">
+        <is>
+          <t>Loading state validado em dispositivo antes do piloto</t>
+        </is>
+      </c>
+      <c r="H23" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Indicadores</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>Visualizar indicadores multidimensionais</t>
+        </is>
+      </c>
+      <c r="D24" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="inlineStr">
+        <is>
+          <t>Vendedor autenticado acessa tela de Indicadores</t>
+        </is>
+      </c>
+      <c r="F24" s="19" t="inlineStr">
+        <is>
+          <t>Cobertura, drop size e positivação com valores reais e metas</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>APK piloto — valores conferidos com Cecília</t>
+        </is>
+      </c>
+      <c r="H24" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="35" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>Remuneração Variável</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>Visualizar RV estimada — perfil representante</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E25" s="21" t="inlineStr">
+        <is>
+          <t>Usuário autenticado com perfil 'representante'</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr">
+        <is>
+          <t>Composição da RV estimada conforme regras validadas</t>
+        </is>
+      </c>
+      <c r="G25" s="21" t="inlineStr">
+        <is>
+          <t>APK piloto — cálculo validado por Cecília</t>
+        </is>
+      </c>
+      <c r="H25" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="35" customHeight="1">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Remuneração Variável</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>Visualizar RV com perfil de supervisor</t>
+        </is>
+      </c>
+      <c r="D26" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>Usuário autenticado com perfil 'supervisor'</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>Indicadores de performance da equipe; diferentes do representante</t>
+        </is>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>Validado em reunião de alinhamento Ago/2025</t>
+        </is>
+      </c>
+      <c r="H26" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="35" customHeight="1">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B27" s="21" t="inlineStr">
+        <is>
+          <t>Pedidos Não Alocados</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>Visualizar lista de pedidos não alocados</t>
+        </is>
+      </c>
+      <c r="D27" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E27" s="21" t="inlineStr">
+        <is>
+          <t>Vendedor autenticado acessa módulo Pedidos N.A.</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="inlineStr">
+        <is>
+          <t>Cards com: nome fantasia, localização, nº pedido, motivo</t>
+        </is>
+      </c>
+      <c r="G27" s="21" t="inlineStr">
+        <is>
+          <t>APK Sprint 1 — validado por Cecília out/2025</t>
+        </is>
+      </c>
+      <c r="H27" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="35" customHeight="1">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>Pedidos Não Alocados</t>
+        </is>
+      </c>
+      <c r="C28" s="19" t="inlineStr">
+        <is>
+          <t>Filtrar pedidos por data e cliente</t>
+        </is>
+      </c>
+      <c r="D28" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="inlineStr">
+        <is>
+          <t>Vendedor aplica filtro na tela de Pedidos N.A.</t>
+        </is>
+      </c>
+      <c r="F28" s="19" t="inlineStr">
+        <is>
+          <t>Lista atualizada com apenas pedidos que correspondem ao filtro</t>
+        </is>
+      </c>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>APK Sprint 1 — validado por Cecília</t>
+        </is>
+      </c>
+      <c r="H28" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="35" customHeight="1">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B29" s="21" t="inlineStr">
+        <is>
+          <t>Pedidos Não Alocados</t>
+        </is>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>Lista vazia de pedidos não alocados</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="E29" s="21" t="inlineStr">
+        <is>
+          <t>Não há pedidos não alocados para o vendedor</t>
+        </is>
+      </c>
+      <c r="F29" s="21" t="inlineStr">
+        <is>
+          <t>Mensagem informativa amigável exibida</t>
+        </is>
+      </c>
+      <c r="G29" s="21" t="inlineStr">
+        <is>
+          <t>Testado com mock de resposta vazia</t>
+        </is>
+      </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="35" customHeight="1">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>Pedidos Não Alocados</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="inlineStr">
+        <is>
+          <t>API retorna formato não padronizado</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>API retorna dados em formato não padronizado</t>
+        </is>
+      </c>
+      <c r="F30" s="19" t="inlineStr">
+        <is>
+          <t>Dados normalizados e exibidos corretamente</t>
+        </is>
+      </c>
+      <c r="G30" s="19" t="inlineStr">
+        <is>
+          <t>Validado durante desenvolvimento Sprint 1</t>
+        </is>
+      </c>
+      <c r="H30" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="35" customHeight="1">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>Visualizar composição da Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E31" s="21" t="inlineStr">
+        <is>
+          <t>Vendedor acessa módulo Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr">
+        <is>
+          <t>Indicadores com progresso real vs. meta; gráficos circulares</t>
+        </is>
+      </c>
+      <c r="G31" s="21" t="inlineStr">
+        <is>
+          <t>APK Sprint 2 — validado por Cecília nov/2025</t>
+        </is>
+      </c>
+      <c r="H31" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="35" customHeight="1">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B32" s="19" t="inlineStr">
+        <is>
+          <t>Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="C32" s="19" t="inlineStr">
+        <is>
+          <t>Pesquisar SKU na Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E32" s="19" t="inlineStr">
+        <is>
+          <t>Vendedor digita SKU no campo de pesquisa</t>
+        </is>
+      </c>
+      <c r="F32" s="19" t="inlineStr">
+        <is>
+          <t>Lista filtrada em tempo real mostrando apenas o SKU pesquisado</t>
+        </is>
+      </c>
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>APK Sprint 2 — testado com lista real</t>
+        </is>
+      </c>
+      <c r="H32" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="35" customHeight="1">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>PDV / Rota PDV</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>Visualizar rota do PDV</t>
+        </is>
+      </c>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E33" s="21" t="inlineStr">
+        <is>
+          <t>Vendedor autenticado acessa módulo Rota PDV</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="inlineStr">
+        <is>
+          <t>Lista de PDVs da rota com status (visitado/pendente)</t>
+        </is>
+      </c>
+      <c r="G33" s="21" t="inlineStr">
+        <is>
+          <t>Validado após recebimento da API (Jan/2026)</t>
+        </is>
+      </c>
+      <c r="H33" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="35" customHeight="1">
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B34" s="19" t="inlineStr">
+        <is>
+          <t>PDV / Rota PDV</t>
+        </is>
+      </c>
+      <c r="C34" s="19" t="inlineStr">
+        <is>
+          <t>Realizar pesquisa de execução de PDV</t>
+        </is>
+      </c>
+      <c r="D34" s="23" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>Vendedor em PDV pendente; GPS ativo</t>
+        </is>
+      </c>
+      <c r="F34" s="19" t="inlineStr">
+        <is>
+          <t>Dados enviados à API; status do PDV muda para 'visitado'</t>
+        </is>
+      </c>
+      <c r="G34" s="19" t="inlineStr">
+        <is>
+          <t>APK Sprint 3 — testado em campo</t>
+        </is>
+      </c>
+      <c r="H34" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="35" customHeight="1">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
+          <t>PDV / Rota PDV</t>
+        </is>
+      </c>
+      <c r="C35" s="21" t="inlineStr">
+        <is>
+          <t>Tentar enviar formulário PDV sem GPS</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="E35" s="21" t="inlineStr">
+        <is>
+          <t>GPS do dispositivo está desativado</t>
+        </is>
+      </c>
+      <c r="F35" s="21" t="inlineStr">
+        <is>
+          <t>Envio bloqueado; mensagem solicita ativação do GPS</t>
+        </is>
+      </c>
+      <c r="G35" s="21" t="inlineStr">
+        <is>
+          <t>Testado com GPS desativado no dispositivo</t>
+        </is>
+      </c>
+      <c r="H35" s="23" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>3. RESUMO DE COBERTURA DE TESTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>Pacote</t>
+        </is>
+      </c>
+      <c r="B39" s="25" t="inlineStr">
+        <is>
+          <t>Total cenários</t>
+        </is>
+      </c>
+      <c r="C39" s="25" t="inlineStr">
+        <is>
+          <t>Happy path</t>
+        </is>
+      </c>
+      <c r="D39" s="25" t="inlineStr">
+        <is>
+          <t>Sad path</t>
+        </is>
+      </c>
+      <c r="E39" s="25" t="inlineStr">
+        <is>
+          <t>Aprovados</t>
+        </is>
+      </c>
+      <c r="F39" s="25" t="inlineStr">
+        <is>
+          <t>Reprovados</t>
+        </is>
+      </c>
+      <c r="G39" s="25" t="inlineStr">
+        <is>
+          <t>% Aprovação</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="26" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B40" s="26" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D40" s="26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E40" s="26" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F40" s="26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G40" s="26" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="27" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B41" s="27" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C41" s="27" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D41" s="27" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G41" s="27" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="28" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C42" s="28" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D42" s="28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E42" s="28" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F42" s="28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G42" s="28" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(FRUKI): expande aba V&V com Gherkin completo (Given/When/Then)
Cada um dos 15 cenários agora exibe colunas separadas Dado / Quando /
Então com o texto Gherkin íntegro extraído de VV-FRUKI01-001 e
VV-FRUKI01-002, incluindo steps com "E" (And).

https://claude.ai/code/session_011KXfcc9u9SbkrrmomU4zNq
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/RAC-FRUKI01-002_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/FTFRUKI_SuperApp-Forca-de-Vendas/RAC-FRUKI01-002_Planilha-de-Gestao-do-Projeto.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,8 +107,28 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00444444"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -190,6 +210,11 @@
         <fgColor rgb="001A5276"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5E8D4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -231,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -315,6 +340,45 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5809,1385 +5873,1033 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>V&amp;V — Cenários de Teste e Evidências · SuperApp Fruki</t>
+          <t>V&amp;V — Cenários de Teste (Gherkin) · SuperApp Fruki · Pacote 1 + Pacote Final 24</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
-        <is>
-          <t>Referências: VV-FRUKI01-001 (Pacote 1) | VV-FRUKI01-002 (Pacote Final 24) | Processo: PRO-VV-001</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
-        <is>
-          <t>1. CICLOS DE EXECUÇÃO</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>Fonte: VV-FRUKI01-001 §6 (Pacote 1) | VV-FRUKI01-002 §6 (Pacote Final 24) | Processo: PRO-VV-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Pacote</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Ciclo</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Módulo / Escopo</t>
-        </is>
-      </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>Itens Verificados</t>
-        </is>
-      </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>Defeitos</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>Resolução</t>
-        </is>
-      </c>
-      <c r="G5" s="16" t="inlineStr">
-        <is>
-          <t>Data</t>
-        </is>
-      </c>
-      <c r="H5" s="16" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Funcionalidade</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>Cenário</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>Dado (Given)</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>Quando (When)</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>Então / E (Then/And)</t>
+        </is>
+      </c>
+      <c r="I3" s="16" t="inlineStr">
+        <is>
+          <t>Evidência</t>
+        </is>
+      </c>
+      <c r="J3" s="16" t="inlineStr">
         <is>
           <t>Situação</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Pacote 1</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
-        <is>
-          <t>Sprint 1 — Desenvolvimento</t>
-        </is>
-      </c>
-      <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>Módulo Metas/RV — telas e APIs</t>
-        </is>
-      </c>
-      <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>RF-01 a RF-04, RNF-01 a RNF-04</t>
-        </is>
-      </c>
-      <c r="E6" s="19" t="inlineStr">
-        <is>
-          <t>2 (duplicação famílias API; latência ~3,10 s)</t>
-        </is>
-      </c>
-      <c r="F6" s="19" t="inlineStr">
-        <is>
-          <t>Tratados no front-end antes do piloto</t>
-        </is>
-      </c>
-      <c r="G6" s="18" t="inlineStr">
-        <is>
-          <t>Jul/2025</t>
-        </is>
-      </c>
-      <c r="H6" s="18" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>Tela de Metas por
+Família de Produtos</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>CT-01</t>
+        </is>
+      </c>
+      <c r="D4" s="32" t="inlineStr">
+        <is>
+          <t>Visualizar metas de volume por família — happy path</t>
+        </is>
+      </c>
+      <c r="E4" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F4" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor está autenticado no SuperApp Fruki</t>
+        </is>
+      </c>
+      <c r="G4" s="34" t="inlineStr">
+        <is>
+          <t>Quando acessa a tela de Metas</t>
+        </is>
+      </c>
+      <c r="H4" s="34" t="inlineStr">
+        <is>
+          <t>Então vê a lista de famílias de produtos ordenada alfabeticamente
+E cada família exibe: volume real, meta do mês e percentual de atingimento
+E os dados refletem o período atual</t>
+        </is>
+      </c>
+      <c r="I4" s="32" t="inlineStr">
+        <is>
+          <t>APK piloto 05/08/2025 — tela validada por Cecília Ribeiro</t>
+        </is>
+      </c>
+      <c r="J4" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>Pacote 1</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>Piloto (vendedores reais)</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>Fluxo completo — Metas, Indicadores, RV</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>Todos os RFs — cenários reais</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>2 (duplicação residual; positivação inconsistente)</t>
-        </is>
-      </c>
-      <c r="F7" s="21" t="inlineStr">
-        <is>
-          <t>Corrigidos antes do aceite (Ago/2025)</t>
-        </is>
-      </c>
-      <c r="G7" s="20" t="inlineStr">
-        <is>
-          <t>05/08/2025</t>
-        </is>
-      </c>
-      <c r="H7" s="20" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Tela de Metas por
+Família de Produtos</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>CT-02</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>API retorna famílias duplicadas — sad path</t>
+        </is>
+      </c>
+      <c r="E5" s="35" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="F5" s="34" t="inlineStr">
+        <is>
+          <t>Dado que a API retorna registros duplicados para uma mesma família</t>
+        </is>
+      </c>
+      <c r="G5" s="34" t="inlineStr">
+        <is>
+          <t>Quando o front-end processa a resposta</t>
+        </is>
+      </c>
+      <c r="H5" s="34" t="inlineStr">
+        <is>
+          <t>Então apenas um registro por família é exibido na tela
+E a ordenação alfabética é mantida</t>
+        </is>
+      </c>
+      <c r="I5" s="32" t="inlineStr">
+        <is>
+          <t>Identificado no piloto; corrigido e revalidado Ago/2025</t>
+        </is>
+      </c>
+      <c r="J5" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Pacote 1</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
-        <is>
-          <t>Revisão de PR — Jardel</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="inlineStr">
-        <is>
-          <t>Código-fonte completo</t>
-        </is>
-      </c>
-      <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>Todos os RFs + código</t>
-        </is>
-      </c>
-      <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F8" s="19" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G8" s="18" t="inlineStr">
-        <is>
-          <t>Ago/2025</t>
-        </is>
-      </c>
-      <c r="H8" s="18" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Tela de Metas por
+Família de Produtos</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="inlineStr">
+        <is>
+          <t>CT-03</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="inlineStr">
+        <is>
+          <t>API demora mais de 3 segundos — sad path</t>
+        </is>
+      </c>
+      <c r="E6" s="35" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="F6" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor acessa a tela de Metas</t>
+        </is>
+      </c>
+      <c r="G6" s="34" t="inlineStr">
+        <is>
+          <t>Quando a resposta da API leva mais de 1 segundo</t>
+        </is>
+      </c>
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>Então um indicador de carregamento (skeleton screen) é exibido
+E os dados aparecem corretamente após o carregamento completo</t>
+        </is>
+      </c>
+      <c r="I6" s="32" t="inlineStr">
+        <is>
+          <t>Loading state validado em dispositivo antes do piloto</t>
+        </is>
+      </c>
+      <c r="J6" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>Pacote 1</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>Aceite final</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>Todos os módulos do Pacote 1</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="inlineStr">
-        <is>
-          <t>Todos os RFs</t>
-        </is>
-      </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F9" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="20" t="inlineStr">
-        <is>
-          <t>Set/2025</t>
-        </is>
-      </c>
-      <c r="H9" s="20" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Indicadores de Cobertura,
+Drop Size e Positivação</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>CT-04</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>Visualizar indicadores multidimensionais — happy path</t>
+        </is>
+      </c>
+      <c r="E7" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F7" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor está autenticado</t>
+        </is>
+      </c>
+      <c r="G7" s="34" t="inlineStr">
+        <is>
+          <t>Quando acessa a tela de Indicadores</t>
+        </is>
+      </c>
+      <c r="H7" s="34" t="inlineStr">
+        <is>
+          <t>Então visualiza cobertura, drop size e positivação com valores reais e metas
+E os cálculos estão de acordo com as regras confirmadas por Cecília Ribeiro</t>
+        </is>
+      </c>
+      <c r="I7" s="32" t="inlineStr">
+        <is>
+          <t>APK piloto — valores conferidos com Cecília Ribeiro</t>
+        </is>
+      </c>
+      <c r="J7" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Remuneração Variável
+(RV) por Perfil</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="inlineStr">
+        <is>
+          <t>CT-05</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="inlineStr">
+        <is>
+          <t>Visualizar RV estimada — perfil "representante" — happy path</t>
+        </is>
+      </c>
+      <c r="E8" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F8" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor está autenticado com perfil "representante"</t>
+        </is>
+      </c>
+      <c r="G8" s="34" t="inlineStr">
+        <is>
+          <t>Quando acessa a tela de RV</t>
+        </is>
+      </c>
+      <c r="H8" s="34" t="inlineStr">
+        <is>
+          <t>Então visualiza a composição da sua RV estimada
+E os indicadores exibidos correspondem ao seu perfil de vendedor
+E o cálculo segue as regras validadas por Cecília Ribeiro</t>
+        </is>
+      </c>
+      <c r="I8" s="32" t="inlineStr">
+        <is>
+          <t>APK piloto — cálculo validado por Cecília Ribeiro</t>
+        </is>
+      </c>
+      <c r="J8" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Pacote 1</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>Remuneração Variável
+(RV) por Perfil</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>CT-06</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>Visualizar RV com perfil de supervisor — happy path</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F9" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o usuário está autenticado com perfil "supervisor"</t>
+        </is>
+      </c>
+      <c r="G9" s="34" t="inlineStr">
+        <is>
+          <t>Quando acessa a tela de Metas</t>
+        </is>
+      </c>
+      <c r="H9" s="34" t="inlineStr">
+        <is>
+          <t>Então visualiza indicadores de performance da sua equipe
+E os dados são diferentes dos indicadores de representante individual</t>
+        </is>
+      </c>
+      <c r="I9" s="32" t="inlineStr">
+        <is>
+          <t>Validado em reunião de alinhamento Ago/2025</t>
+        </is>
+      </c>
+      <c r="J9" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="36" t="inlineStr">
         <is>
           <t>Pacote Final 24</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>Sprint 1</t>
-        </is>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>Pedidos Não Alocados</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>RF-05 a RF-08</t>
-        </is>
-      </c>
-      <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>1 (formato não padronizado da API de pedidos)</t>
-        </is>
-      </c>
-      <c r="F10" s="19" t="inlineStr">
-        <is>
-          <t>Normalização em pedidosNaoAlocadosService.ts</t>
-        </is>
-      </c>
-      <c r="G10" s="18" t="inlineStr">
-        <is>
-          <t>Out/2025</t>
-        </is>
-      </c>
-      <c r="H10" s="18" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="B10" s="36" t="inlineStr">
+        <is>
+          <t>Módulo Pedidos
+Não Alocados</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>CT-07</t>
+        </is>
+      </c>
+      <c r="D10" s="32" t="inlineStr">
+        <is>
+          <t>Visualizar lista de pedidos não alocados — happy path</t>
+        </is>
+      </c>
+      <c r="E10" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F10" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor está autenticado no SuperApp Fruki</t>
+        </is>
+      </c>
+      <c r="G10" s="34" t="inlineStr">
+        <is>
+          <t>Quando acessa o módulo Pedidos Não Alocados</t>
+        </is>
+      </c>
+      <c r="H10" s="34" t="inlineStr">
+        <is>
+          <t>Então vê cards com: nome fantasia do cliente, localização, número do pedido e motivo de não alocação
+E os dados são carregados da API</t>
+        </is>
+      </c>
+      <c r="I10" s="32" t="inlineStr">
+        <is>
+          <t>APK Sprint 1 — validado por Cecília Ribeiro out/2025</t>
+        </is>
+      </c>
+      <c r="J10" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="36" t="inlineStr">
         <is>
           <t>Pacote Final 24</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
-        <is>
-          <t>Revisão PR #57</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="inlineStr">
-        <is>
-          <t>Módulo Pedidos Não Alocados — código</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>Padrões, performance, autenticação</t>
-        </is>
-      </c>
-      <c r="E11" s="21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F11" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="20" t="inlineStr">
-        <is>
-          <t>25/10/2025</t>
-        </is>
-      </c>
-      <c r="H11" s="20" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
+        <is>
+          <t>Módulo Pedidos
+Não Alocados</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>CT-08</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>Filtrar pedidos por data e cliente — happy path</t>
+        </is>
+      </c>
+      <c r="E11" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F11" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor está na tela de Pedidos Não Alocados</t>
+        </is>
+      </c>
+      <c r="G11" s="34" t="inlineStr">
+        <is>
+          <t>Quando aplica filtro por período ou cliente</t>
+        </is>
+      </c>
+      <c r="H11" s="34" t="inlineStr">
+        <is>
+          <t>Então a lista é atualizada exibindo apenas os pedidos que correspondem ao filtro</t>
+        </is>
+      </c>
+      <c r="I11" s="32" t="inlineStr">
+        <is>
+          <t>APK Sprint 1 — validado por Cecília Ribeiro</t>
+        </is>
+      </c>
+      <c r="J11" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="52" customHeight="1">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t>Pacote Final 24</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="inlineStr">
-        <is>
-          <t>Regra de Ouro</t>
-        </is>
-      </c>
-      <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>RF-09 a RF-11</t>
-        </is>
-      </c>
-      <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="inlineStr">
-        <is>
-          <t>Módulo entregue conforme protótipo</t>
-        </is>
-      </c>
-      <c r="G12" s="18" t="inlineStr">
-        <is>
-          <t>Nov/2025</t>
-        </is>
-      </c>
-      <c r="H12" s="18" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="B12" s="36" t="inlineStr">
+        <is>
+          <t>Módulo Pedidos
+Não Alocados</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>CT-09</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>Lista vazia de pedidos não alocados — sad path</t>
+        </is>
+      </c>
+      <c r="E12" s="35" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="F12" s="34" t="inlineStr">
+        <is>
+          <t>Dado que não há pedidos não alocados para o vendedor</t>
+        </is>
+      </c>
+      <c r="G12" s="34" t="inlineStr">
+        <is>
+          <t>Quando acessa o módulo Pedidos Não Alocados</t>
+        </is>
+      </c>
+      <c r="H12" s="34" t="inlineStr">
+        <is>
+          <t>Então uma mensagem informativa amigável é exibida</t>
+        </is>
+      </c>
+      <c r="I12" s="32" t="inlineStr">
+        <is>
+          <t>Testado com mock de resposta vazia</t>
+        </is>
+      </c>
+      <c r="J12" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="52" customHeight="1">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>Pacote Final 24</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
-        <is>
-          <t>Revisão PR — Regra de Ouro</t>
-        </is>
-      </c>
-      <c r="C13" s="21" t="inlineStr">
-        <is>
-          <t>Código do módulo Regra de Ouro</t>
-        </is>
-      </c>
-      <c r="D13" s="21" t="inlineStr">
-        <is>
-          <t>Padrões, performance, integração</t>
-        </is>
-      </c>
-      <c r="E13" s="21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F13" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="inlineStr">
-        <is>
-          <t>Nov/2025</t>
-        </is>
-      </c>
-      <c r="H13" s="20" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="B13" s="36" t="inlineStr">
+        <is>
+          <t>Módulo Pedidos
+Não Alocados</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>CT-10</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>API retorna formato não padronizado — sad path</t>
+        </is>
+      </c>
+      <c r="E13" s="35" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="F13" s="34" t="inlineStr">
+        <is>
+          <t>Dado que a API de pedidos não alocados retorna dados em formato não padronizado</t>
+        </is>
+      </c>
+      <c r="G13" s="34" t="inlineStr">
+        <is>
+          <t>Quando o front-end processa a resposta</t>
+        </is>
+      </c>
+      <c r="H13" s="34" t="inlineStr">
+        <is>
+          <t>Então os dados são normalizados e exibidos corretamente na tela</t>
+        </is>
+      </c>
+      <c r="I13" s="32" t="inlineStr">
+        <is>
+          <t>Validado durante desenvolvimento Sprint 1</t>
+        </is>
+      </c>
+      <c r="J13" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="52" customHeight="1">
+      <c r="A14" s="36" t="inlineStr">
         <is>
           <t>Pacote Final 24</t>
         </is>
       </c>
-      <c r="B14" s="18" t="inlineStr">
-        <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>PDV / Rota PDV</t>
-        </is>
-      </c>
-      <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>RF-12 a RF-14</t>
-        </is>
-      </c>
-      <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>1 (API Rota PDV recebida só em 08/01/2026)</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="inlineStr">
-        <is>
-          <t>Desenvolvimento paralelo da UI; integração Jan/2026</t>
-        </is>
-      </c>
-      <c r="G14" s="18" t="inlineStr">
-        <is>
-          <t>Dez/2025–Jan/2026</t>
-        </is>
-      </c>
-      <c r="H14" s="18" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>Módulo Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>CT-11</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>Visualizar composição da Regra de Ouro — happy path</t>
+        </is>
+      </c>
+      <c r="E14" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor está autenticado</t>
+        </is>
+      </c>
+      <c r="G14" s="34" t="inlineStr">
+        <is>
+          <t>Quando acessa o módulo Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>Então vê todos os indicadores da Regra de Ouro com progresso real vs. meta
+E gráficos circulares distinguem indicadores acima e abaixo da meta</t>
+        </is>
+      </c>
+      <c r="I14" s="32" t="inlineStr">
+        <is>
+          <t>APK Sprint 2 — validado por Cecília Ribeiro nov/2025</t>
+        </is>
+      </c>
+      <c r="J14" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="36" t="inlineStr">
         <is>
           <t>Pacote Final 24</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
-        <is>
-          <t>Build AAB v2.0</t>
-        </is>
-      </c>
-      <c r="C15" s="21" t="inlineStr">
-        <is>
-          <t>Todos os módulos — build de produção</t>
-        </is>
-      </c>
-      <c r="D15" s="21" t="inlineStr">
-        <is>
-          <t>RNF-01, RNF-03</t>
-        </is>
-      </c>
-      <c r="E15" s="21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F15" s="21" t="inlineStr">
-        <is>
-          <t>AAB gerado e entregue para publicação</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
-        <is>
-          <t>Jan/2026</t>
-        </is>
-      </c>
-      <c r="H15" s="20" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="B15" s="36" t="inlineStr">
+        <is>
+          <t>Módulo Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>CT-12</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>Pesquisar SKU na Regra de Ouro — happy path</t>
+        </is>
+      </c>
+      <c r="E15" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor está na tela Regra de Ouro</t>
+        </is>
+      </c>
+      <c r="G15" s="34" t="inlineStr">
+        <is>
+          <t>Quando digita um SKU no campo de pesquisa</t>
+        </is>
+      </c>
+      <c r="H15" s="34" t="inlineStr">
+        <is>
+          <t>Então a lista de indicadores é filtrada em tempo real mostrando apenas o SKU pesquisado</t>
+        </is>
+      </c>
+      <c r="I15" s="32" t="inlineStr">
+        <is>
+          <t>APK Sprint 2 — testado com lista real</t>
+        </is>
+      </c>
+      <c r="J15" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="36" t="inlineStr">
         <is>
           <t>Pacote Final 24</t>
         </is>
       </c>
-      <c r="B16" s="18" t="inlineStr">
-        <is>
-          <t>Aceite final</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="inlineStr">
-        <is>
-          <t>Todos os módulos do PF24</t>
-        </is>
-      </c>
-      <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>RF-05 a RF-14</t>
-        </is>
-      </c>
-      <c r="E16" s="19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F16" s="19" t="inlineStr">
-        <is>
-          <t>Aceite formal via Microsoft Teams</t>
-        </is>
-      </c>
-      <c r="G16" s="18" t="inlineStr">
-        <is>
-          <t>15/01/2026</t>
-        </is>
-      </c>
-      <c r="H16" s="18" t="inlineStr">
-        <is>
-          <t>✅ Concluído</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>2. CENÁRIOS DE TESTE — RESULTADOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="B16" s="36" t="inlineStr">
+        <is>
+          <t>Módulo PDV /
+Rota PDV</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>CT-13</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
+        <is>
+          <t>Visualizar rota do PDV — happy path</t>
+        </is>
+      </c>
+      <c r="E16" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor está autenticado</t>
+        </is>
+      </c>
+      <c r="G16" s="34" t="inlineStr">
+        <is>
+          <t>Quando acessa o módulo Rota PDV</t>
+        </is>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>Então vê a lista de PDVs da sua rota com status (visitado/pendente)</t>
+        </is>
+      </c>
+      <c r="I16" s="32" t="inlineStr">
+        <is>
+          <t>Validado após recebimento da API (Jan/2026)</t>
+        </is>
+      </c>
+      <c r="J16" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="36" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B17" s="36" t="inlineStr">
+        <is>
+          <t>Módulo PDV /
+Rota PDV</t>
+        </is>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>CT-14</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>Realizar pesquisa de execução de PDV com geolocalização — happy path</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o vendedor está em um PDV pendente
+E o GPS está ativo e a geolocalização foi capturada</t>
+        </is>
+      </c>
+      <c r="G17" s="34" t="inlineStr">
+        <is>
+          <t>Quando acessa o formulário de pesquisa, responde todas as perguntas e confirma o envio</t>
+        </is>
+      </c>
+      <c r="H17" s="34" t="inlineStr">
+        <is>
+          <t>Então os dados são enviados para a API de Rota PDV com sucesso
+E o status do PDV muda para "visitado"</t>
+        </is>
+      </c>
+      <c r="I17" s="32" t="inlineStr">
+        <is>
+          <t>APK Sprint 3 — testado em campo</t>
+        </is>
+      </c>
+      <c r="J17" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="36" t="inlineStr">
+        <is>
+          <t>Pacote Final 24</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="inlineStr">
+        <is>
+          <t>Módulo PDV /
+Rota PDV</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>CT-15</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <t>Tentar enviar formulário PDV sem GPS — sad path</t>
+        </is>
+      </c>
+      <c r="E18" s="35" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="F18" s="34" t="inlineStr">
+        <is>
+          <t>Dado que o GPS do dispositivo está desativado</t>
+        </is>
+      </c>
+      <c r="G18" s="34" t="inlineStr">
+        <is>
+          <t>Quando tenta enviar o formulário de pesquisa de PDV</t>
+        </is>
+      </c>
+      <c r="H18" s="34" t="inlineStr">
+        <is>
+          <t>Então o envio é bloqueado
+E uma mensagem solicita a ativação do GPS para validar a presença</t>
+        </is>
+      </c>
+      <c r="I18" s="32" t="inlineStr">
+        <is>
+          <t>Testado com GPS desativado no dispositivo</t>
+        </is>
+      </c>
+      <c r="J18" s="33" t="inlineStr">
+        <is>
+          <t>✅ Aprovado</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>RESUMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="38" t="inlineStr">
         <is>
           <t>Pacote</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
-        <is>
-          <t>Módulo</t>
-        </is>
-      </c>
-      <c r="C20" s="16" t="inlineStr">
-        <is>
-          <t>Cenário</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>Pré-condição / Ação</t>
-        </is>
-      </c>
-      <c r="F20" s="16" t="inlineStr">
-        <is>
-          <t>Resultado Esperado</t>
-        </is>
-      </c>
-      <c r="G20" s="16" t="inlineStr">
-        <is>
-          <t>Evidência</t>
-        </is>
-      </c>
-      <c r="H20" s="16" t="inlineStr">
-        <is>
-          <t>Situação</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="35" customHeight="1">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t>Total CT</t>
+        </is>
+      </c>
+      <c r="C22" s="38" t="inlineStr">
+        <is>
+          <t>Happy</t>
+        </is>
+      </c>
+      <c r="D22" s="38" t="inlineStr">
+        <is>
+          <t>Sad</t>
+        </is>
+      </c>
+      <c r="E22" s="38" t="inlineStr">
+        <is>
+          <t>Aprovados</t>
+        </is>
+      </c>
+      <c r="F22" s="38" t="inlineStr">
+        <is>
+          <t>% Aprovação</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="39" t="inlineStr">
         <is>
           <t>Pacote 1</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
-        <is>
-          <t>Metas por Família</t>
-        </is>
-      </c>
-      <c r="C21" s="21" t="inlineStr">
-        <is>
-          <t>Visualizar metas de volume por família</t>
-        </is>
-      </c>
-      <c r="D21" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E21" s="21" t="inlineStr">
-        <is>
-          <t>Vendedor autenticado acessa tela de Metas</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="inlineStr">
-        <is>
-          <t>Lista de famílias c/ volume real, meta e % atingimento</t>
-        </is>
-      </c>
-      <c r="G21" s="21" t="inlineStr">
-        <is>
-          <t>APK piloto 05/08/2025 — validado por Cecília</t>
-        </is>
-      </c>
-      <c r="H21" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="35" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
-        <is>
-          <t>Pacote 1</t>
-        </is>
-      </c>
-      <c r="B22" s="19" t="inlineStr">
-        <is>
-          <t>Metas por Família</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="inlineStr">
-        <is>
-          <t>API retorna famílias duplicadas</t>
-        </is>
-      </c>
-      <c r="D22" s="24" t="inlineStr">
-        <is>
-          <t>Sad</t>
-        </is>
-      </c>
-      <c r="E22" s="19" t="inlineStr">
-        <is>
-          <t>API retorna registros duplicados para mesma família</t>
-        </is>
-      </c>
-      <c r="F22" s="19" t="inlineStr">
-        <is>
-          <t>Apenas um registro por família exibido; ordenação mantida</t>
-        </is>
-      </c>
-      <c r="G22" s="19" t="inlineStr">
-        <is>
-          <t>Identificado no piloto; corrigido e revalidado Ago/2025</t>
-        </is>
-      </c>
-      <c r="H22" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="35" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>Pacote 1</t>
-        </is>
-      </c>
-      <c r="B23" s="21" t="inlineStr">
-        <is>
-          <t>Metas por Família</t>
-        </is>
-      </c>
-      <c r="C23" s="21" t="inlineStr">
-        <is>
-          <t>API demora mais de 3 segundos</t>
-        </is>
-      </c>
-      <c r="D23" s="24" t="inlineStr">
-        <is>
-          <t>Sad</t>
-        </is>
-      </c>
-      <c r="E23" s="21" t="inlineStr">
-        <is>
-          <t>Resposta da API leva mais de 1 segundo</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="inlineStr">
-        <is>
-          <t>Skeleton screen exibido; dados aparecem após carregamento</t>
-        </is>
-      </c>
-      <c r="G23" s="21" t="inlineStr">
-        <is>
-          <t>Loading state validado em dispositivo antes do piloto</t>
-        </is>
-      </c>
-      <c r="H23" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="35" customHeight="1">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>Pacote 1</t>
-        </is>
-      </c>
-      <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>Indicadores</t>
-        </is>
-      </c>
-      <c r="C24" s="19" t="inlineStr">
-        <is>
-          <t>Visualizar indicadores multidimensionais</t>
-        </is>
-      </c>
-      <c r="D24" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E24" s="19" t="inlineStr">
-        <is>
-          <t>Vendedor autenticado acessa tela de Indicadores</t>
-        </is>
-      </c>
-      <c r="F24" s="19" t="inlineStr">
-        <is>
-          <t>Cobertura, drop size e positivação com valores reais e metas</t>
-        </is>
-      </c>
-      <c r="G24" s="19" t="inlineStr">
-        <is>
-          <t>APK piloto — valores conferidos com Cecília</t>
-        </is>
-      </c>
-      <c r="H24" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="35" customHeight="1">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>Pacote 1</t>
-        </is>
-      </c>
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>Remuneração Variável</t>
-        </is>
-      </c>
-      <c r="C25" s="21" t="inlineStr">
-        <is>
-          <t>Visualizar RV estimada — perfil representante</t>
-        </is>
-      </c>
-      <c r="D25" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E25" s="21" t="inlineStr">
-        <is>
-          <t>Usuário autenticado com perfil 'representante'</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="inlineStr">
-        <is>
-          <t>Composição da RV estimada conforme regras validadas</t>
-        </is>
-      </c>
-      <c r="G25" s="21" t="inlineStr">
-        <is>
-          <t>APK piloto — cálculo validado por Cecília</t>
-        </is>
-      </c>
-      <c r="H25" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="35" customHeight="1">
-      <c r="A26" s="17" t="inlineStr">
-        <is>
-          <t>Pacote 1</t>
-        </is>
-      </c>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>Remuneração Variável</t>
-        </is>
-      </c>
-      <c r="C26" s="19" t="inlineStr">
-        <is>
-          <t>Visualizar RV com perfil de supervisor</t>
-        </is>
-      </c>
-      <c r="D26" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E26" s="19" t="inlineStr">
-        <is>
-          <t>Usuário autenticado com perfil 'supervisor'</t>
-        </is>
-      </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>Indicadores de performance da equipe; diferentes do representante</t>
-        </is>
-      </c>
-      <c r="G26" s="19" t="inlineStr">
-        <is>
-          <t>Validado em reunião de alinhamento Ago/2025</t>
-        </is>
-      </c>
-      <c r="H26" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="35" customHeight="1">
-      <c r="A27" s="22" t="inlineStr">
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E23" s="39" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F23" s="39" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="40" t="inlineStr">
         <is>
           <t>Pacote Final 24</t>
         </is>
       </c>
-      <c r="B27" s="21" t="inlineStr">
-        <is>
-          <t>Pedidos Não Alocados</t>
-        </is>
-      </c>
-      <c r="C27" s="21" t="inlineStr">
-        <is>
-          <t>Visualizar lista de pedidos não alocados</t>
-        </is>
-      </c>
-      <c r="D27" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E27" s="21" t="inlineStr">
-        <is>
-          <t>Vendedor autenticado acessa módulo Pedidos N.A.</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="inlineStr">
-        <is>
-          <t>Cards com: nome fantasia, localização, nº pedido, motivo</t>
-        </is>
-      </c>
-      <c r="G27" s="21" t="inlineStr">
-        <is>
-          <t>APK Sprint 1 — validado por Cecília out/2025</t>
-        </is>
-      </c>
-      <c r="H27" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="35" customHeight="1">
-      <c r="A28" s="22" t="inlineStr">
-        <is>
-          <t>Pacote Final 24</t>
-        </is>
-      </c>
-      <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>Pedidos Não Alocados</t>
-        </is>
-      </c>
-      <c r="C28" s="19" t="inlineStr">
-        <is>
-          <t>Filtrar pedidos por data e cliente</t>
-        </is>
-      </c>
-      <c r="D28" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E28" s="19" t="inlineStr">
-        <is>
-          <t>Vendedor aplica filtro na tela de Pedidos N.A.</t>
-        </is>
-      </c>
-      <c r="F28" s="19" t="inlineStr">
-        <is>
-          <t>Lista atualizada com apenas pedidos que correspondem ao filtro</t>
-        </is>
-      </c>
-      <c r="G28" s="19" t="inlineStr">
-        <is>
-          <t>APK Sprint 1 — validado por Cecília</t>
-        </is>
-      </c>
-      <c r="H28" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="35" customHeight="1">
-      <c r="A29" s="22" t="inlineStr">
-        <is>
-          <t>Pacote Final 24</t>
-        </is>
-      </c>
-      <c r="B29" s="21" t="inlineStr">
-        <is>
-          <t>Pedidos Não Alocados</t>
-        </is>
-      </c>
-      <c r="C29" s="21" t="inlineStr">
-        <is>
-          <t>Lista vazia de pedidos não alocados</t>
-        </is>
-      </c>
-      <c r="D29" s="24" t="inlineStr">
-        <is>
-          <t>Sad</t>
-        </is>
-      </c>
-      <c r="E29" s="21" t="inlineStr">
-        <is>
-          <t>Não há pedidos não alocados para o vendedor</t>
-        </is>
-      </c>
-      <c r="F29" s="21" t="inlineStr">
-        <is>
-          <t>Mensagem informativa amigável exibida</t>
-        </is>
-      </c>
-      <c r="G29" s="21" t="inlineStr">
-        <is>
-          <t>Testado com mock de resposta vazia</t>
-        </is>
-      </c>
-      <c r="H29" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="35" customHeight="1">
-      <c r="A30" s="22" t="inlineStr">
-        <is>
-          <t>Pacote Final 24</t>
-        </is>
-      </c>
-      <c r="B30" s="19" t="inlineStr">
-        <is>
-          <t>Pedidos Não Alocados</t>
-        </is>
-      </c>
-      <c r="C30" s="19" t="inlineStr">
-        <is>
-          <t>API retorna formato não padronizado</t>
-        </is>
-      </c>
-      <c r="D30" s="24" t="inlineStr">
-        <is>
-          <t>Sad</t>
-        </is>
-      </c>
-      <c r="E30" s="19" t="inlineStr">
-        <is>
-          <t>API retorna dados em formato não padronizado</t>
-        </is>
-      </c>
-      <c r="F30" s="19" t="inlineStr">
-        <is>
-          <t>Dados normalizados e exibidos corretamente</t>
-        </is>
-      </c>
-      <c r="G30" s="19" t="inlineStr">
-        <is>
-          <t>Validado durante desenvolvimento Sprint 1</t>
-        </is>
-      </c>
-      <c r="H30" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="35" customHeight="1">
-      <c r="A31" s="22" t="inlineStr">
-        <is>
-          <t>Pacote Final 24</t>
-        </is>
-      </c>
-      <c r="B31" s="21" t="inlineStr">
-        <is>
-          <t>Regra de Ouro</t>
-        </is>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>Visualizar composição da Regra de Ouro</t>
-        </is>
-      </c>
-      <c r="D31" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E31" s="21" t="inlineStr">
-        <is>
-          <t>Vendedor acessa módulo Regra de Ouro</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr">
-        <is>
-          <t>Indicadores com progresso real vs. meta; gráficos circulares</t>
-        </is>
-      </c>
-      <c r="G31" s="21" t="inlineStr">
-        <is>
-          <t>APK Sprint 2 — validado por Cecília nov/2025</t>
-        </is>
-      </c>
-      <c r="H31" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="35" customHeight="1">
-      <c r="A32" s="22" t="inlineStr">
-        <is>
-          <t>Pacote Final 24</t>
-        </is>
-      </c>
-      <c r="B32" s="19" t="inlineStr">
-        <is>
-          <t>Regra de Ouro</t>
-        </is>
-      </c>
-      <c r="C32" s="19" t="inlineStr">
-        <is>
-          <t>Pesquisar SKU na Regra de Ouro</t>
-        </is>
-      </c>
-      <c r="D32" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E32" s="19" t="inlineStr">
-        <is>
-          <t>Vendedor digita SKU no campo de pesquisa</t>
-        </is>
-      </c>
-      <c r="F32" s="19" t="inlineStr">
-        <is>
-          <t>Lista filtrada em tempo real mostrando apenas o SKU pesquisado</t>
-        </is>
-      </c>
-      <c r="G32" s="19" t="inlineStr">
-        <is>
-          <t>APK Sprint 2 — testado com lista real</t>
-        </is>
-      </c>
-      <c r="H32" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="35" customHeight="1">
-      <c r="A33" s="22" t="inlineStr">
-        <is>
-          <t>Pacote Final 24</t>
-        </is>
-      </c>
-      <c r="B33" s="21" t="inlineStr">
-        <is>
-          <t>PDV / Rota PDV</t>
-        </is>
-      </c>
-      <c r="C33" s="21" t="inlineStr">
-        <is>
-          <t>Visualizar rota do PDV</t>
-        </is>
-      </c>
-      <c r="D33" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E33" s="21" t="inlineStr">
-        <is>
-          <t>Vendedor autenticado acessa módulo Rota PDV</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr">
-        <is>
-          <t>Lista de PDVs da rota com status (visitado/pendente)</t>
-        </is>
-      </c>
-      <c r="G33" s="21" t="inlineStr">
-        <is>
-          <t>Validado após recebimento da API (Jan/2026)</t>
-        </is>
-      </c>
-      <c r="H33" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="35" customHeight="1">
-      <c r="A34" s="22" t="inlineStr">
-        <is>
-          <t>Pacote Final 24</t>
-        </is>
-      </c>
-      <c r="B34" s="19" t="inlineStr">
-        <is>
-          <t>PDV / Rota PDV</t>
-        </is>
-      </c>
-      <c r="C34" s="19" t="inlineStr">
-        <is>
-          <t>Realizar pesquisa de execução de PDV</t>
-        </is>
-      </c>
-      <c r="D34" s="23" t="inlineStr">
-        <is>
-          <t>Happy</t>
-        </is>
-      </c>
-      <c r="E34" s="19" t="inlineStr">
-        <is>
-          <t>Vendedor em PDV pendente; GPS ativo</t>
-        </is>
-      </c>
-      <c r="F34" s="19" t="inlineStr">
-        <is>
-          <t>Dados enviados à API; status do PDV muda para 'visitado'</t>
-        </is>
-      </c>
-      <c r="G34" s="19" t="inlineStr">
-        <is>
-          <t>APK Sprint 3 — testado em campo</t>
-        </is>
-      </c>
-      <c r="H34" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="35" customHeight="1">
-      <c r="A35" s="22" t="inlineStr">
-        <is>
-          <t>Pacote Final 24</t>
-        </is>
-      </c>
-      <c r="B35" s="21" t="inlineStr">
-        <is>
-          <t>PDV / Rota PDV</t>
-        </is>
-      </c>
-      <c r="C35" s="21" t="inlineStr">
-        <is>
-          <t>Tentar enviar formulário PDV sem GPS</t>
-        </is>
-      </c>
-      <c r="D35" s="24" t="inlineStr">
-        <is>
-          <t>Sad</t>
-        </is>
-      </c>
-      <c r="E35" s="21" t="inlineStr">
-        <is>
-          <t>GPS do dispositivo está desativado</t>
-        </is>
-      </c>
-      <c r="F35" s="21" t="inlineStr">
-        <is>
-          <t>Envio bloqueado; mensagem solicita ativação do GPS</t>
-        </is>
-      </c>
-      <c r="G35" s="21" t="inlineStr">
-        <is>
-          <t>Testado com GPS desativado no dispositivo</t>
-        </is>
-      </c>
-      <c r="H35" s="23" t="inlineStr">
-        <is>
-          <t>✅ Aprovado</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="15" t="inlineStr">
-        <is>
-          <t>3. RESUMO DE COBERTURA DE TESTES</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="25" t="inlineStr">
-        <is>
-          <t>Pacote</t>
-        </is>
-      </c>
-      <c r="B39" s="25" t="inlineStr">
-        <is>
-          <t>Total cenários</t>
-        </is>
-      </c>
-      <c r="C39" s="25" t="inlineStr">
-        <is>
-          <t>Happy path</t>
-        </is>
-      </c>
-      <c r="D39" s="25" t="inlineStr">
-        <is>
-          <t>Sad path</t>
-        </is>
-      </c>
-      <c r="E39" s="25" t="inlineStr">
-        <is>
-          <t>Aprovados</t>
-        </is>
-      </c>
-      <c r="F39" s="25" t="inlineStr">
-        <is>
-          <t>Reprovados</t>
-        </is>
-      </c>
-      <c r="G39" s="25" t="inlineStr">
-        <is>
-          <t>% Aprovação</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="26" t="inlineStr">
-        <is>
-          <t>Pacote 1</t>
-        </is>
-      </c>
-      <c r="B40" s="26" t="inlineStr">
+      <c r="B24" s="40" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C24" s="40" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C40" s="26" t="inlineStr">
+      <c r="D24" s="40" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E24" s="40" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F24" s="40" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B25" s="41" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D25" s="41" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D40" s="26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E40" s="26" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="F40" s="26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G40" s="26" t="inlineStr">
+      <c r="E25" s="41" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F25" s="41" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="27" t="inlineStr">
-        <is>
-          <t>Pacote Final 24</t>
-        </is>
-      </c>
-      <c r="B41" s="27" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="C41" s="27" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D41" s="27" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E41" s="27" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="F41" s="27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G41" s="27" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="28" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B42" s="28" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="C42" s="28" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="D42" s="28" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E42" s="28" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="F42" s="28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G42" s="28" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A1:H1"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A21:J21"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>